<commit_message>
Mark import template data as test data pending review
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/importacion/plantilla-importacion-CC-001-Rev3.xlsx
+++ b/docs/importacion/plantilla-importacion-CC-001-Rev3.xlsx
@@ -1546,7 +1546,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <cols>
     <col min="1" max="1" width="58.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -1562,119 +1562,127 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Proyecto destino (propuesto)</v>
+        <v>Estado de los datos</v>
       </c>
       <c r="B2" t="str">
-        <v>CC-001 Rev. 3 (8 oct 2026)</v>
+        <v>DATOS DE PRUEBA: supuestos confirmados por el equipo; las fechas pasarán por una revisión antes de uso real</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Fecha de inicio del proyecto (supuesto)</v>
+        <v>Proyecto destino (propuesto)</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-10-19</v>
+        <v>CC-001 Rev. 3 (8 oct 2026)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Días hábiles</v>
+        <v>Fecha de inicio del proyecto (supuesto)</v>
       </c>
       <c r="B4" t="str">
-        <v>Lunes a viernes, sin feriados (hoja Feriados)</v>
+        <v>2026-10-19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Calendario de feriados</v>
+        <v>Días hábiles</v>
       </c>
       <c r="B5" t="str">
-        <v>Guatemala (supuesto, por confirmar)</v>
+        <v>Lunes a viernes, sin feriados (hoja Feriados)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Pruebas entre tareas</v>
+        <v>Calendario de feriados</v>
       </c>
       <c r="B6" t="str">
-        <v>2 días hábiles entre el fin de una tarea y el inicio de la siguiente del mismo hito</v>
+        <v>Guatemala (supuesto, por confirmar)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Encadenamiento</v>
+        <v>Pruebas entre tareas</v>
       </c>
       <c r="B7" t="str">
-        <v>Las tareas de un hito van en secuencia; los hitos corren en paralelo</v>
+        <v>2 días hábiles entre el fin de una tarea y el inicio de la siguiente del mismo hito</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Orden dentro del hito</v>
+        <v>Encadenamiento</v>
       </c>
       <c r="B8" t="str">
-        <v>Decisión funcional → Dependencia externa → Desarrollo → Documentación → Aprobación comercial</v>
+        <v>Las tareas de un hito van en secuencia; los hitos corren en paralelo</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Duración por tipo (días hábiles, incluye el día de inicio)</v>
+        <v>Orden dentro del hito</v>
       </c>
       <c r="B9" t="str">
-        <v>Decisión funcional: 3; Dependencia externa: 5; Desarrollo: 5; Documentación: 2; Aprobación comercial: 3</v>
+        <v>Decisión funcional → Dependencia externa → Desarrollo → Documentación → Aprobación comercial</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Hitos con tareas</v>
+        <v>Duración por tipo (días hábiles, incluye el día de inicio)</v>
       </c>
       <c r="B10" t="str">
-        <v>10: CC-C04, CC-C10, CC-C03, CC-C11, CC-C01, CC-C02, CC-C08, CC-C07, CC-M01, CC-C13</v>
+        <v>Decisión funcional: 3; Dependencia externa: 5; Desarrollo: 5; Documentación: 2; Aprobación comercial: 3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Hitos del PDF sin tareas</v>
+        <v>Hitos con tareas</v>
       </c>
       <c r="B11" t="str">
-        <v>CC-C09 y CC-C12: ninguna tarea los cita como primer código, así que no se crean hasta que tengan tareas</v>
+        <v>10: CC-C04, CC-C10, CC-C03, CC-C11, CC-C01, CC-C02, CC-C08, CC-C07, CC-M01, CC-C13</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Tarea con varios CC</v>
+        <v>Hitos del PDF sin tareas</v>
       </c>
       <c r="B12" t="str">
-        <v>Se asigna solo al primer código; los originales están en la hoja Referencia</v>
+        <v>CC-C09 y CC-C12: ninguna tarea los cita como primer código, así que no se crean hasta que tengan tareas</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Tareas sin CC</v>
+        <v>Tarea con varios CC</v>
       </c>
       <c r="B13" t="str">
-        <v>Quedan fuera (5): pendientes de decidir a qué hito se asignan</v>
+        <v>Se asigna solo al primer código; los originales están en la hoja Referencia</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Responsable</v>
+        <v>Tareas sin CC</v>
       </c>
       <c r="B14" t="str">
-        <v>Vacío: los documentos no lo confirman</v>
+        <v>Quedan fuera (5): pendientes de decidir a qué hito se asignan</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>Responsable</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Vacío: los documentos no lo confirman</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Fin del último hito</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
         <v>2026-11-17</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add CC-GEN milestone for tasks without a change control and dev plan
Group the five tasks that no change control backs under a general
milestone in the import template (28 tasks, 11 milestones), and document
the local development plan for F01.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/importacion/plantilla-importacion-CC-001-Rev3.xlsx
+++ b/docs/importacion/plantilla-importacion-CC-001-Rev3.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G29"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -965,16 +965,131 @@
         <v>46317</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Gestión contractual y transversal del CC-001 Rev. 3</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Tareas del análisis de Lucalza que no pertenecen a ningún control de cambio del documento: correcciones fuera del alcance de los CC, condiciones de pago y plazo, y actualización del documento de diseño.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Cerrar por escrito el alcance de la vista de seguimiento para supervisores e Inside Sales</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" s="1">
+        <v>46314</v>
+      </c>
+      <c r="G25" s="1">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Gestión contractual y transversal del CC-001 Rev. 3</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Tareas del análisis de Lucalza que no pertenecen a ningún control de cambio del documento: correcciones fuera del alcance de los CC, condiciones de pago y plazo, y actualización del documento de diseño.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Revisar y corregir la sincronización de contactos con SAP (creación, edición y eliminación)</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" s="1">
+        <v>46322</v>
+      </c>
+      <c r="G26" s="1">
+        <v>46328</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Gestión contractual y transversal del CC-001 Rev. 3</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Tareas del análisis de Lucalza que no pertenecen a ningún control de cambio del documento: correcciones fuera del alcance de los CC, condiciones de pago y plazo, y actualización del documento de diseño.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Actualizar el documento de diseño y arquitectura antes de la firma</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" s="1">
+        <v>46331</v>
+      </c>
+      <c r="G27" s="1">
+        <v>46332</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Gestión contractual y transversal del CC-001 Rev. 3</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Tareas del análisis de Lucalza que no pertenecen a ningún control de cambio del documento: correcciones fuera del alcance de los CC, condiciones de pago y plazo, y actualización del documento de diseño.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Acordar el pago por hitos en lugar del 100 % a la firma</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" s="1">
+        <v>46337</v>
+      </c>
+      <c r="G28" s="1">
+        <v>46339</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Gestión contractual y transversal del CC-001 Rev. 3</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Tareas del análisis de Lucalza que no pertenecen a ningún control de cambio del documento: correcciones fuera del alcance de los CC, condiciones de pago y plazo, y actualización del documento de diseño.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Cerrar el cronograma y las dependencias de Lucalza con fecha y responsable</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" s="1">
+        <v>46344</v>
+      </c>
+      <c r="G29" s="1">
+        <v>46346</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G29"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -1537,9 +1652,124 @@
         <v>El requisito 2 prohíbe elegir bodega y el 3 permite escribir el código; tras sincronizar se valida y se avisa al supervisor. Faltan plazo y responsable del flujo de excepción. El análisis registra que se indicó que sí pueden generar la lista de bodegas.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Cerrar por escrito el alcance de la vista de seguimiento para supervisores e Inside Sales</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Decisión funcional</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v>Hallazgo 16; Revisión: sin control de cambio</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Requiere filtros por vendedor, supervisor y país, reglas Farmer y Hunter, días desde la última compra y respetar la ruta configurada. Según el análisis, Freeway aceptó una customización completa en la revisión del diseño y la minuta del 19 de agosto.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Revisar y corregir la sincronización de contactos con SAP (creación, edición y eliminación)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Desarrollo</v>
+      </c>
+      <c r="D26">
+        <v>5</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v>Hallazgo 9; Revisión: sin control de cambio</v>
+      </c>
+      <c r="G26" t="str">
+        <v>En las pruebas solo sincronizan nombre, teléfono y correo; ningún control de cambio lo cubre. Se pide corrección sin costo y con fecha.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Actualizar el documento de diseño y arquitectura antes de la firma</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Documentación</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v>Hallazgo 27</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Pendiente desde la minuta del 19 de agosto; el CC lo cita como fuente única (págs. 44 y 52).</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Acordar el pago por hitos en lugar del 100 % a la firma</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Aprobación comercial</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>Hallazgo 25; Revisión: Documentos</v>
+      </c>
+      <c r="G28" t="str">
+        <v>V3 (pág. 52) pide USD 51,271 a la firma. El análisis propone una parte a la firma, otra con las pruebas listas y el resto tras la aceptación y el soporte; es una propuesta, no un acuerdo.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>CC-GEN</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Cerrar el cronograma y las dependencias de Lucalza con fecha y responsable</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Aprobación comercial</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>Hallazgo 26</v>
+      </c>
+      <c r="G29" t="str">
+        <v>V3 propone construcción del 8 de octubre al 27 de noviembre, pruebas del 30 de noviembre al 4 de diciembre y producción el 11 de diciembre, sujetas a ajustes. Son fechas propuestas por Freeway, no aprobadas, y no se usan como fechas del hito. Se pide que un cambio de fechas no suba el precio.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1637,7 +1867,7 @@
         <v>Hitos con tareas</v>
       </c>
       <c r="B11" t="str">
-        <v>10: CC-C04, CC-C10, CC-C03, CC-C11, CC-C01, CC-C02, CC-C08, CC-C07, CC-M01, CC-C13</v>
+        <v>11: CC-C04, CC-C10, CC-C03, CC-C11, CC-C01, CC-C02, CC-C08, CC-C07, CC-GEN, CC-M01, CC-C13</v>
       </c>
     </row>
     <row r="12">
@@ -1661,7 +1891,7 @@
         <v>Tareas sin CC</v>
       </c>
       <c r="B14" t="str">
-        <v>Quedan fuera (5): pendientes de decidir a qué hito se asignan</v>
+        <v>Las 5 tareas sin control de cambio van al hito CC-GEN (código marcador, no es un CC del PDF)</v>
       </c>
     </row>
     <row r="15">
@@ -1677,7 +1907,7 @@
         <v>Fin del último hito</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-11-17</v>
+        <v>2026-11-20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>